<commit_message>
added 2 ways for check
</commit_message>
<xml_diff>
--- a/worklog.xlsx
+++ b/worklog.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,6 +453,26 @@
           <t>end_time</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>checkin_date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>expected_end_time</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>checkout_date</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>checkout_time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -473,6 +493,10 @@
       <c r="D2" s="2" t="n">
         <v>46172.05264996528</v>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -495,6 +519,10 @@
           <t>01:30</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -517,6 +545,10 @@
           <t>01:40</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -539,6 +571,10 @@
           <t>01:50</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -561,6 +597,10 @@
           <t>01:55</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -581,6 +621,90 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>01:55</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>17:20</t>
         </is>
       </c>
     </row>

</xml_diff>